<commit_message>
V3.0 ana sürüm: büyük güncellemeler ve yeni özellikler
</commit_message>
<xml_diff>
--- a/data/iasi/service_status.xlsx
+++ b/data/iasi/service_status.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:H64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1370,8 +1370,6 @@
           <t>Servis</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr">
         <is>
           <t>Toplu servise alındı</t>
@@ -1383,6 +1381,1096 @@
         </is>
       </c>
       <c r="H30" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2217</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>2026-04-15 15:23:38</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2218</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>2026-04-15 15:23:38</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2219</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>2026-04-15 15:23:39</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2220</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>2026-04-15 15:23:39</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2221</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>2026-04-15 15:23:39</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>2222</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>2026-04-15 15:23:39</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>2223</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>2026-04-15 15:23:39</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>2224</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>2026-04-15 15:23:40</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>2225</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>2026-04-15 15:23:40</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>2226</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>2026-04-15 15:23:40</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>2227</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>2026-04-15 15:23:40</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>2228</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>2026-04-15 15:23:40</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>2229</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>2026-04-15 15:23:41</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>2230</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>2026-04-15 15:23:41</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>2231</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>2026-04-15 15:23:42</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>2232</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>2026-04-15 15:23:42</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>2233</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>2026-04-15 15:23:42</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>2234</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>2026-04-15 15:23:42</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>2235</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>2026-04-15 15:23:42</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>2236</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>2026-04-15 15:23:43</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>2237</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>2026-04-15 15:23:43</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>2238</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>2026-04-15 15:23:43</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>2239</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>2026-04-15 15:23:43</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>2240</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>2026-04-15 15:23:43</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>2241</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>2026-04-15 15:23:43</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>2242</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>2026-04-15 15:23:44</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>2243</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>2026-04-15 15:23:44</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>2244</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>2026-04-15 15:23:44</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>2245</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>2026-04-15 15:23:44</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>2246</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>2026-04-15 15:23:44</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>2247</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>2026-04-15 15:23:45</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>2248</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>2026-04-15 15:23:45</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>2249</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>2026-04-15 15:23:45</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>2250</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" t="inlineStr"/>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>2026-04-15 15:23:45</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
         <is>
           <t>admin</t>
         </is>

</xml_diff>